<commit_message>
10/03/2026 - Observaciones atendidas
</commit_message>
<xml_diff>
--- a/plantillas/consulta/Validacion_Resultados.xlsx
+++ b/plantillas/consulta/Validacion_Resultados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Visual Studio Code\NodeJS\SIVACC\plantillas\consulta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B20E85F-455F-4EA8-B3E5-0A5F7EB39C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C83D9212-E53C-432F-B79F-4F56573E9D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 (Las marcadas con la palabra "voto" en la Lista nominal y las que opinaron con resoluciones del Tribunal Electoral)</t>
   </si>
   <si>
-    <t>Total de personas que votaron
+    <t>Total de personas que emitieron su opinión
 (EN CASO DE ACTAS LEVANTADAS EN DIRECCIÓN DISTRITAL)</t>
   </si>
 </sst>

</xml_diff>